<commit_message>
docs(trazabilidad): crear registro único de identificadores y alinear matriz
</commit_message>
<xml_diff>
--- a/datos/trazabilidad/matriz-trazabilidad.xlsx
+++ b/datos/trazabilidad/matriz-trazabilidad.xlsx
@@ -482,7 +482,7 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Evento EV</t>
+          <t>Evento (INT)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
@@ -519,7 +519,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>EV-01</t>
+          <t>INT-01/EV-03</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -556,7 +556,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>EV-02</t>
+          <t>INT-01/EV-05</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -593,7 +593,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>EV-03</t>
+          <t>INT-01/EV-06, EV-10</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -630,7 +630,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>EV-04</t>
+          <t>INT-01/EV-09</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -667,7 +667,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>EV-05</t>
+          <t>INT-01/EV-11</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -704,7 +704,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>EV-06</t>
+          <t>Por definir (ERP)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -741,7 +741,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>EV-07</t>
+          <t>Por definir (ERP)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -778,7 +778,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>EV-08</t>
+          <t>Por definir (ERP)</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>EV-09</t>
+          <t>Por definir (ERP)</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>EV-10</t>
+          <t>Por definir (ERP)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -889,7 +889,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>EV-11</t>
+          <t>Por definir (ERP)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="13.8"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1018,17 +1018,17 @@
     <row r="1" ht="34.05" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Regla RN</t>
+          <t>Regla (RN/EXC)</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Evento EV</t>
+          <t>Evento (INT)</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Control CT</t>
+          <t>Control (CT/SOD)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>EV-01</t>
+          <t>INT-01/EV-03</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>EV-02</t>
+          <t>INT-01/EV-05</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -1117,7 +1117,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>CP-01 / CP-02</t>
+          <t>CP-01</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -1127,12 +1127,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Contexto de la empresa / Flujo O2C</t>
+          <t>Decisiones comerciales</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Identificar cliente según necesidad de la transacción y mantener origen del dato.</t>
+          <t>Toda oportunidad abierta tiene próxima acción, fecha y responsable.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1144,17 +1144,17 @@
     <row r="4" ht="69" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>RN-03</t>
+          <t>RN-03 / RN-04</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>EV-03</t>
+          <t>INT-01/EV-06, EV-10</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>CT-03</t>
+          <t>CT-03 / CT-04</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -1186,17 +1186,17 @@
     <row r="5" ht="69" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>RN-04</t>
+          <t>EXC-01</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>EV-04</t>
+          <t>INT-01/EV-08, EV-09</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>CT-04</t>
+          <t>SOD-01</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -1228,37 +1228,37 @@
     <row r="6" ht="69" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>RN-05 / RN-P2-01</t>
+          <t>RN-05</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>EV-03 / EV-05</t>
+          <t>INT-01/EV-07</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>CT-05 / CT-P2-01</t>
+          <t>CT-05</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>CP-01 / CP-02</t>
+          <t>CP-01</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>TR-03 / TR-05</t>
+          <t>TR-03</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Flujo O2C / C4 componentes ventas</t>
+          <t>Decisiones comerciales</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Vincular aceptación del cliente con cotización y pedido; conservar versión.</t>
+          <t>Solo personal autorizado confirma disponibilidad o fecha al cliente.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -1270,37 +1270,37 @@
     <row r="7" ht="69" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>RN-06 / RN-P2-02</t>
+          <t>RN-06</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>EV-06</t>
+          <t>INT-01/EV-06</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>CT-06 / CT-P2-02</t>
+          <t>CT-06</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>CP-01 / CP-02</t>
+          <t>CP-01</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>TR-06</t>
+          <t>TR-03</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Flujo de inventario / C4 componentes inventario</t>
+          <t>Decisiones comerciales</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Relacionar pedido y reserva con disponibilidad por ubicación.</t>
+          <t>Registrar el comprobante previsto sin exigir RUC para cotizar.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -1312,17 +1312,17 @@
     <row r="8" ht="69" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>RN-P2-03</t>
+          <t>RN-07</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>EV-07</t>
+          <t>INT-01/EV-11</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>CT-P2-03</t>
+          <t>CT-07</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -1332,17 +1332,17 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>TR-07</t>
+          <t>TR-02 / TR-05</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Flujo de inventario / C4 componentes inventario</t>
+          <t>Contexto de la empresa / Flujo O2C</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Conservar cantidades realmente entregadas y diferencias físicas.</t>
+          <t>Identificar cliente según necesidad de la transacción y mantener origen del dato.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -1354,17 +1354,17 @@
     <row r="9" ht="69" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>RN-P2-04</t>
+          <t>RN-08</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>EV-08</t>
+          <t>INT-01/EV-11</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>CT-P2-04</t>
+          <t>CT-08</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -1374,17 +1374,17 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>TR-08</t>
+          <t>TR-05</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Contexto de la empresa / C4 contexto</t>
+          <t>Flujo O2C / C4 componentes ventas</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Conciliar referencia fiscal KeyFacil con pedido y valores correspondientes.</t>
+          <t>Vincular aceptación del cliente con cotización y pedido; conservar versión.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -1396,37 +1396,37 @@
     <row r="10" ht="69" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>RN-P2-05</t>
+          <t>RN-09</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>EV-09</t>
+          <t>Por definir (ERP)</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>CT-P2-05</t>
+          <t>CT-09</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>CP-01</t>
+          <t>CP-01 / CP-02</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>TR-09</t>
+          <t>TR-06</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Contexto de la empresa / Flujo O2C</t>
+          <t>Flujo de inventario / C4 componentes inventario</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Documentar cada cobro verificable y el saldo restante.</t>
+          <t>Relacionar pedido y reserva con disponibilidad por ubicación.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1438,17 +1438,17 @@
     <row r="11" ht="69" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>RN-P2-06</t>
+          <t>RN-10</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>EV-10</t>
+          <t>Por definir (ERP)</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>CT-P2-06</t>
+          <t>CT-10</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -1458,17 +1458,17 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>TR-10</t>
+          <t>TR-07</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Extensión futura (posventa)</t>
+          <t>Flujo de inventario / C4 componentes inventario</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Relacionar caso de atención posterior con pedido de origen.</t>
+          <t>Conservar cantidades realmente entregadas y diferencias físicas.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1480,37 +1480,37 @@
     <row r="12" ht="69" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>RN-P2-07</t>
+          <t>RN-11</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>EV-11</t>
+          <t>Por definir (ERP)</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>CT-P2-07</t>
+          <t>CT-11</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>CP-01</t>
+          <t>CP-01 / CP-02</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>TR-11</t>
+          <t>TR-08</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Riesgos y controles / Flujo O2C</t>
+          <t>Contexto de la empresa / C4 contexto</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Verificar cierre con entrega, cobro, incidencias y conformidad requerida.</t>
+          <t>Conciliar referencia fiscal KeyFacil con pedido y valores correspondientes.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1522,40 +1522,166 @@
     <row r="13" ht="69" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>RN-07</t>
+          <t>RN-12</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>EV-05</t>
+          <t>Por definir (ERP)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>CT-07</t>
+          <t>CT-12</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
+          <t>CP-01</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>TR-09</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Contexto de la empresa / Flujo O2C</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Documentar cada cobro verificable y el saldo restante.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Control propuesto · CP planificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>RN-13</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Por definir (ERP)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>CT-13</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>CP-01 / CP-02</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>TR-10</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Extensión futura (posventa)</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Relacionar caso de atención posterior con pedido de origen.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Control propuesto · CP planificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>RN-14</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Por definir (ERP)</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>CT-14</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>CP-01</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>TR-11</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Riesgos y controles / Flujo O2C</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Verificar cierre con entrega, cobro, incidencias y conformidad requerida.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Control propuesto · CP planificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>RN-15</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Por definir (ERP)</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>CT-15</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
           <t>CP-02</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>TR-05</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Contexto de la empresa (crédito actual)</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Registrar decisión expresa de condiciones de crédito por propietario.</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Control propuesto · CP planificado</t>
         </is>
@@ -1634,12 +1760,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Abrir `CORR-2026-0042` [SIM]; anotar entorno, usuario auditor y fecha.</t>
+          <t>Abrir el caso por `OPP-SIM-001` [SIM] (cuenta `CLI-SIM-001`); anotar entorno, usuario auditor y fecha.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Índice de referencias; a documentar en prueba.</t>
+          <t>Cadena de identificadores del catálogo sintético.</t>
         </is>
       </c>
       <c r="E2" s="2" t="n"/>
@@ -1692,7 +1818,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Abrir `COT-2026-0042`, versiones, líneas, precio y aceptación.</t>
+          <t>Abrir `COT-SIM-001-V01`, versiones, líneas, precio y aceptación.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -1750,7 +1876,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Seguir `SO-2026-0042` desde aceptación; revisar respuesta y llave de reintento si existe interfaz.</t>
+          <t>Seguir el pedido `PED-SIM-001` [SIM] desde la aceptación, cuando exista; revisar respuesta y llave de reintento si existe interfaz.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -1808,7 +1934,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Comparar pedido, `F001-004512` [SIM] en KeyFacil, monto y pago por separado.</t>
+          <t>Comparar pedido, comprobante `CPE-SIM-001` [SIM] en KeyFacil, monto y pago por separado.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1866,7 +1992,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Comprobar correlación, secuencia de tiempos, cambios antes/después, accesos y huecos.</t>
+          <t>Comprobar la cadena de identificadores, secuencia de tiempos, cambios antes/después, accesos y huecos.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">

</xml_diff>